<commit_message>
2026-05-13 docs+dev: 주간보고/개발현황/ONBOARDING 갱신 + BOM 부모 추출 스크립트
- 주간보고.md: 이번 주 작업 범위 (Phase B 부서 결재 + 입출고 v2 UX) 반영
- 개발현황.xlsx: 재생성
- ONBOARDING.md: '창고입출고' 표기 띄어쓰기 통일
- scripts/dev/extract_io_bom_parents.py: 입출고 관리대장 xlsx 에서 BOM 부모 후보 추출 유틸

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/개발현황.xlsx
+++ b/docs/개발현황.xlsx
@@ -552,7 +552,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -568,46 +568,58 @@
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>개발 기간</t>
+          <t>개발 기간 (회사)</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>2026-04-10 ~ 05-08 (29일 · 근무일 18일)</t>
+          <t>2026-04-21 ~ 05-08 (18일 · 근무일 11일)</t>
         </is>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>총 커밋 수</t>
+          <t>개인 선행 작업</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>355건</t>
+          <t>2026-04-10 ~ 04-20 (회사 개발 착수 이전 · 개인 시간)</t>
         </is>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>기능 완료</t>
+          <t>총 커밋 수</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>41 / 51개 (80%)</t>
+          <t>391건 (회사 기간 287건)</t>
         </is>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
+          <t>기능 완료</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>41 / 51개 (80%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
           <t>개발 영역</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Backend · Frontend · Mobile · Admin · Docs</t>
         </is>
@@ -777,12 +789,26 @@
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>2026-05-08  ■■■■■■■  (14)</t>
+          <t>2026-05-08  ■■■■■■■■■■■■■  (26)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="18" customHeight="1">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-11  ■■■■■■■■  (16)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="18" customHeight="1">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-12  ■■■■  (8)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="29">
+  <mergeCells count="32">
     <mergeCell ref="A30:E30"/>
     <mergeCell ref="A24:E24"/>
     <mergeCell ref="A15:E15"/>
@@ -793,13 +819,16 @@
     <mergeCell ref="B4:E4"/>
     <mergeCell ref="A16:E16"/>
     <mergeCell ref="A25:E25"/>
+    <mergeCell ref="B7:E7"/>
     <mergeCell ref="B3:E3"/>
     <mergeCell ref="A18:E18"/>
     <mergeCell ref="A27:E27"/>
     <mergeCell ref="A21:E21"/>
     <mergeCell ref="A12:E12"/>
     <mergeCell ref="A26:E26"/>
+    <mergeCell ref="A33:E33"/>
     <mergeCell ref="A23:E23"/>
+    <mergeCell ref="A32:E32"/>
     <mergeCell ref="A14:E14"/>
     <mergeCell ref="A8:E8"/>
     <mergeCell ref="A22:E22"/>
@@ -868,7 +897,7 @@
       </c>
       <c r="B2" s="7" t="inlineStr">
         <is>
-          <t>기반 구축</t>
+          <t>기반 구축 (개인 선행)</t>
         </is>
       </c>
       <c r="C2" s="8" t="inlineStr">
@@ -893,7 +922,7 @@
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>UI 개발</t>
+          <t>UI 개발 (개인 선행)</t>
         </is>
       </c>
       <c r="C3" s="8" t="inlineStr">
@@ -919,7 +948,7 @@
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>기능 고도화</t>
+          <t>기능 고도화 (개인 선행)</t>
         </is>
       </c>
       <c r="C4" s="8" t="inlineStr">
@@ -945,7 +974,7 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>UI 정제</t>
+          <t>UI 정제 (회사 개발 착수)</t>
         </is>
       </c>
       <c r="C5" s="8" t="inlineStr">
@@ -1063,7 +1092,7 @@
         </is>
       </c>
       <c r="D9" s="7" t="n">
-        <v>124</v>
+        <v>136</v>
       </c>
       <c r="E9" s="9" t="inlineStr">
         <is>
@@ -2313,7 +2342,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D24"/>
+  <dimension ref="A1:D26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2869,7 +2898,7 @@
         </is>
       </c>
       <c r="B24" s="16" t="n">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="C24" s="17" t="inlineStr">
         <is>
@@ -2881,6 +2910,54 @@
         </is>
       </c>
       <c r="D24" s="16" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="50" customHeight="1">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="n">
+        <v>16</v>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-11 docs: 데스크톱 전체 화면 스크린샷 캡처 (라이트모드)
+2026-05-11 docs: BOM 세팅 도구 조립+진공 합본 698건 프리셋 임베드
+2026-05-11 docs: BOM 세팅 도구 고압 99건 추가 합본 796건 + DB 동기화
+2026-05-11 admin: 관리자 화면 UI/UX 전면 정리 (PIN/8개 섹션/BOM 가로분할)
+Implement warehouse IO v2</t>
+        </is>
+      </c>
+      <c r="D25" s="7" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="50" customHeight="1">
+      <c r="A26" s="16" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="B26" s="16" t="n">
+        <v>8</v>
+      </c>
+      <c r="C26" s="17" t="inlineStr">
+        <is>
+          <t>2026-05-12 frontend: 입출고 v2 compose UX 정리 (NavFooter 제거 · 컬럼
+2026-05-12 fix: .dev/*.log gitignore 추가 (dev 서버 stdout 덤프 노이
+2026-05-12 backend+frontend: 생산 가능 immediate/maximum 정의 재정의 
+2026-05-12 frontend: 로그인 단일 카드 재구성 (3단계 → 콤보박스+PIN 1화면)
+2026-05-12 dev: 빌드 디렉터리 분리 (.next-prod) + dev 재시작 헬퍼</t>
+        </is>
+      </c>
+      <c r="D26" s="16" t="inlineStr">
         <is>
           <t>Frontend</t>
         </is>
@@ -2897,7 +2974,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D356"/>
+  <dimension ref="A1:D392"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -10738,6 +10815,798 @@
         </is>
       </c>
     </row>
+    <row r="357">
+      <c r="A357" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="B357" s="7" t="inlineStr">
+        <is>
+          <t>3a281ac</t>
+        </is>
+      </c>
+      <c r="C357" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-08 fix: docs/openapi.json baseline 갱신 (CI drift 해소)</t>
+        </is>
+      </c>
+      <c r="D357" s="7" t="inlineStr">
+        <is>
+          <t>fix</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" s="16" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="B358" s="16" t="inlineStr">
+        <is>
+          <t>32980ef</t>
+        </is>
+      </c>
+      <c r="C358" s="17" t="inlineStr">
+        <is>
+          <t>2026-05-08 desktop: 주간보고 디자인 다듬기 (가독성/색구분/컬럼분배)</t>
+        </is>
+      </c>
+      <c r="D358" s="16" t="inlineStr">
+        <is>
+          <t>desktop</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="B359" s="7" t="inlineStr">
+        <is>
+          <t>aa0d626</t>
+        </is>
+      </c>
+      <c r="C359" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-08 desktop: 부서 재고 조정 양방향 진행 + 탭 자동 새로고침 제거</t>
+        </is>
+      </c>
+      <c r="D359" s="7" t="inlineStr">
+        <is>
+          <t>desktop</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" s="16" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="B360" s="16" t="inlineStr">
+        <is>
+          <t>85b2cb2</t>
+        </is>
+      </c>
+      <c r="C360" s="17" t="inlineStr">
+        <is>
+          <t>2026-05-08 backend: erp.db UUID 형식 정규화 마이그레이션 스크립트</t>
+        </is>
+      </c>
+      <c r="D360" s="16" t="inlineStr">
+        <is>
+          <t>backend</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="B361" s="7" t="inlineStr">
+        <is>
+          <t>7ad0dfa</t>
+        </is>
+      </c>
+      <c r="C361" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-08 docs: 주간보고/개발현황 5/8 갱신</t>
+        </is>
+      </c>
+      <c r="D361" s="7" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" s="16" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="B362" s="16" t="inlineStr">
+        <is>
+          <t>174387e</t>
+        </is>
+      </c>
+      <c r="C362" s="17" t="inlineStr">
+        <is>
+          <t>2026-05-08 backend: 30명 동시 입출고 운영 안정성 보강</t>
+        </is>
+      </c>
+      <c r="D362" s="16" t="inlineStr">
+        <is>
+          <t>backend</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="B363" s="7" t="inlineStr">
+        <is>
+          <t>681e9e2</t>
+        </is>
+      </c>
+      <c r="C363" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-08 ops: 30명 실사용 기준 동시 입출고 안정성 완성</t>
+        </is>
+      </c>
+      <c r="D363" s="7" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" s="16" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="B364" s="16" t="inlineStr">
+        <is>
+          <t>aca3a4b</t>
+        </is>
+      </c>
+      <c r="C364" s="17" t="inlineStr">
+        <is>
+          <t>2026-05-08 ops: 30명 실사용 기준 안정성 80점 이상 보강</t>
+        </is>
+      </c>
+      <c r="D364" s="16" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="B365" s="7" t="inlineStr">
+        <is>
+          <t>24eab65</t>
+        </is>
+      </c>
+      <c r="C365" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-08 ops: 30명 실사용 전 항목 90점 안정성 보강</t>
+        </is>
+      </c>
+      <c r="D365" s="7" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" s="16" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="B366" s="16" t="inlineStr">
+        <is>
+          <t>28127f6</t>
+        </is>
+      </c>
+      <c r="C366" s="17" t="inlineStr">
+        <is>
+          <t>2026-05-08 ops: 30명 실사용 안정성 100점 검증 완성</t>
+        </is>
+      </c>
+      <c r="D366" s="16" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="B367" s="7" t="inlineStr">
+        <is>
+          <t>596457c</t>
+        </is>
+      </c>
+      <c r="C367" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-08 frontend: 컴포넌트 재사용성 리팩터링 (Phase 1)</t>
+        </is>
+      </c>
+      <c r="D367" s="7" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" s="16" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="B368" s="16" t="inlineStr">
+        <is>
+          <t>8bedf79</t>
+        </is>
+      </c>
+      <c r="C368" s="17" t="inlineStr">
+        <is>
+          <t>2026-05-08 frontend: 컴포넌트 재사용성 리팩터링 (Phase 2-3)</t>
+        </is>
+      </c>
+      <c r="D368" s="16" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="B369" s="7" t="inlineStr">
+        <is>
+          <t>c3f0810</t>
+        </is>
+      </c>
+      <c r="C369" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-11 docs: 데스크톱 전체 화면 스크린샷 캡처 (라이트모드)</t>
+        </is>
+      </c>
+      <c r="D369" s="7" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" s="16" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="B370" s="16" t="inlineStr">
+        <is>
+          <t>89a38c0</t>
+        </is>
+      </c>
+      <c r="C370" s="17" t="inlineStr">
+        <is>
+          <t>2026-05-11 docs: BOM 세팅 도구 조립+진공 합본 698건 프리셋 임베드</t>
+        </is>
+      </c>
+      <c r="D370" s="16" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="B371" s="7" t="inlineStr">
+        <is>
+          <t>1947a97</t>
+        </is>
+      </c>
+      <c r="C371" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-11 docs: BOM 세팅 도구 고압 99건 추가 합본 796건 + DB 동기화</t>
+        </is>
+      </c>
+      <c r="D371" s="7" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" s="16" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="B372" s="16" t="inlineStr">
+        <is>
+          <t>183f0ef</t>
+        </is>
+      </c>
+      <c r="C372" s="17" t="inlineStr">
+        <is>
+          <t>2026-05-11 admin: 관리자 화면 UI/UX 전면 정리 (PIN/8개 섹션/BOM 가로분할)</t>
+        </is>
+      </c>
+      <c r="D372" s="16" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="B373" s="7" t="inlineStr">
+        <is>
+          <t>8518c73</t>
+        </is>
+      </c>
+      <c r="C373" s="8" t="inlineStr">
+        <is>
+          <t>Implement warehouse IO v2</t>
+        </is>
+      </c>
+      <c r="D373" s="7" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" s="16" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="B374" s="16" t="inlineStr">
+        <is>
+          <t>308d85e</t>
+        </is>
+      </c>
+      <c r="C374" s="17" t="inlineStr">
+        <is>
+          <t>Update OpenAPI schema baseline</t>
+        </is>
+      </c>
+      <c r="D374" s="16" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="B375" s="7" t="inlineStr">
+        <is>
+          <t>8914a31</t>
+        </is>
+      </c>
+      <c r="C375" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-11 frontend: 입출고 v2 마법사 UX 보정 + 작업유형 권한 가드</t>
+        </is>
+      </c>
+      <c r="D375" s="7" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" s="16" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="B376" s="16" t="inlineStr">
+        <is>
+          <t>045c405</t>
+        </is>
+      </c>
+      <c r="C376" s="17" t="inlineStr">
+        <is>
+          <t>2026-05-11 docs: BOM 세팅 도구 튜닝(NF) 9건 추가 805건</t>
+        </is>
+      </c>
+      <c r="D376" s="16" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="B377" s="7" t="inlineStr">
+        <is>
+          <t>0e49d78</t>
+        </is>
+      </c>
+      <c r="C377" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-11 frontend: 대시보드 필터 정비 + 관리자 KPI 카드 컴팩트화</t>
+        </is>
+      </c>
+      <c r="D377" s="7" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" s="16" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="B378" s="16" t="inlineStr">
+        <is>
+          <t>c22671e</t>
+        </is>
+      </c>
+      <c r="C378" s="17" t="inlineStr">
+        <is>
+          <t>2026-05-11 fix: openapi baseline 갱신 (입출고 초안 submit 엔드포인트)</t>
+        </is>
+      </c>
+      <c r="D378" s="16" t="inlineStr">
+        <is>
+          <t>fix</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="B379" s="7" t="inlineStr">
+        <is>
+          <t>b3316ad</t>
+        </is>
+      </c>
+      <c r="C379" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-11 merge: feat/frontend-ux-overhaul x claude/show-branch-commits-sgEQD</t>
+        </is>
+      </c>
+      <c r="D379" s="7" t="inlineStr">
+        <is>
+          <t>merge</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" s="16" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="B380" s="16" t="inlineStr">
+        <is>
+          <t>5e7b05e</t>
+        </is>
+      </c>
+      <c r="C380" s="17" t="inlineStr">
+        <is>
+          <t>2026-05-11 fix: openapi baseline 갱신 (client_request_id 멱등 키 필드)</t>
+        </is>
+      </c>
+      <c r="D380" s="16" t="inlineStr">
+        <is>
+          <t>fix</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="B381" s="7" t="inlineStr">
+        <is>
+          <t>ea3b29d</t>
+        </is>
+      </c>
+      <c r="C381" s="8" t="inlineStr">
+        <is>
+          <t>Merge pull request #14 from Hw-03/merge/ux-overhaul-x-ops-hardening</t>
+        </is>
+      </c>
+      <c r="D381" s="7" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" s="16" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="B382" s="16" t="inlineStr">
+        <is>
+          <t>8a2e5af</t>
+        </is>
+      </c>
+      <c r="C382" s="17" t="inlineStr">
+        <is>
+          <t>2026-05-11 backend+frontend: 입출고 v2 client_request_id 멱등성 + 409/503 UX</t>
+        </is>
+      </c>
+      <c r="D382" s="16" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="B383" s="7" t="inlineStr">
+        <is>
+          <t>4d249b9</t>
+        </is>
+      </c>
+      <c r="C383" s="8" t="inlineStr">
+        <is>
+          <t>Merge pull request #15 from Hw-03/feat/io-v2-idempotency</t>
+        </is>
+      </c>
+      <c r="D383" s="7" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" s="16" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="B384" s="16" t="inlineStr">
+        <is>
+          <t>7a4a08f</t>
+        </is>
+      </c>
+      <c r="C384" s="17" t="inlineStr">
+        <is>
+          <t>Merge pull request #16 from Hw-03/feat/frontend-ux-overhaul</t>
+        </is>
+      </c>
+      <c r="D384" s="16" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="B385" s="7" t="inlineStr">
+        <is>
+          <t>8e16069</t>
+        </is>
+      </c>
+      <c r="C385" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-12 frontend: 입출고 v2 compose UX 정리 (NavFooter 제거 · 컬럼 분리 · 자동 advance)</t>
+        </is>
+      </c>
+      <c r="D385" s="7" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" s="16" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="B386" s="16" t="inlineStr">
+        <is>
+          <t>b900a02</t>
+        </is>
+      </c>
+      <c r="C386" s="17" t="inlineStr">
+        <is>
+          <t>2026-05-12 fix: .dev/*.log gitignore 추가 (dev 서버 stdout 덤프 노이즈 제거)</t>
+        </is>
+      </c>
+      <c r="D386" s="16" t="inlineStr">
+        <is>
+          <t>fix</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="B387" s="7" t="inlineStr">
+        <is>
+          <t>7bb4c8e</t>
+        </is>
+      </c>
+      <c r="C387" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-12 backend+frontend: 생산 가능 immediate/maximum 정의 재정의 + status 4분기 표시</t>
+        </is>
+      </c>
+      <c r="D387" s="7" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" s="16" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="B388" s="16" t="inlineStr">
+        <is>
+          <t>c5df180</t>
+        </is>
+      </c>
+      <c r="C388" s="17" t="inlineStr">
+        <is>
+          <t>2026-05-12 frontend: 로그인 단일 카드 재구성 (3단계 → 콤보박스+PIN 1화면)</t>
+        </is>
+      </c>
+      <c r="D388" s="16" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="B389" s="7" t="inlineStr">
+        <is>
+          <t>d33976a</t>
+        </is>
+      </c>
+      <c r="C389" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-12 dev: 빌드 디렉터리 분리 (.next-prod) + dev 재시작 헬퍼</t>
+        </is>
+      </c>
+      <c r="D389" s="7" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" s="16" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="B390" s="16" t="inlineStr">
+        <is>
+          <t>3bf456f</t>
+        </is>
+      </c>
+      <c r="C390" s="17" t="inlineStr">
+        <is>
+          <t>2026-05-12 fix: next 14 --distDir CLI 미지원 → next.config.js phase 분기로 전환</t>
+        </is>
+      </c>
+      <c r="D390" s="16" t="inlineStr">
+        <is>
+          <t>fix</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="B391" s="7" t="inlineStr">
+        <is>
+          <t>b6244ae</t>
+        </is>
+      </c>
+      <c r="C391" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-12 frontend+backend: 입출고 v2 sub_type 기반 버튼/태그 + 수량보정 입고/출고 분리</t>
+        </is>
+      </c>
+      <c r="D391" s="7" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" s="16" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="B392" s="16" t="inlineStr">
+        <is>
+          <t>faeebc3</t>
+        </is>
+      </c>
+      <c r="C392" s="17" t="inlineStr">
+        <is>
+          <t>2026-05-12 frontend: 셀렉트 디자인 통일 (AppSelect) + 입출고 v2 부서 입출고/BOM 가드/수량 보정</t>
+        </is>
+      </c>
+      <c r="D392" s="16" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
2026-05-15 docs: 주간보고 5/9~5/15 + 개발현황 엑셀 갱신
- 주간보고: 입출고 v2 4단계 마법사·멱등성·위저드 재디자인,
  부서 결재 + 직원 권한 분리, BOM 805건 입력 진행, 재고 이미지 컬럼,
  데이터 모델 정리(legacy 제거), 개발 환경/CI 정비
- 개발현황 엑셀:
  - KPI를 회사 개발 기간(2026-04-21~05-15, 25일·근무일 16일)과
    개인 선행 작업(2026-04-10~04-20)으로 분리 표기
  - Sheet 2 5/9~5/15 행 추가, 4/10~4/19 항목에 (개인 선행) 라벨
  - 신규 기능 10종 반영, 기능 완료 53/62 (85%)

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/개발현황.xlsx
+++ b/docs/개발현황.xlsx
@@ -552,7 +552,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -573,7 +573,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>2026-04-21 ~ 05-08 (18일 · 근무일 11일)</t>
+          <t>2026-04-21 ~ 05-15 (25일 · 근무일 16일)</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>391건 (회사 기간 287건)</t>
+          <t>421건 (회사 기간 341건)</t>
         </is>
       </c>
     </row>
@@ -609,7 +609,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>41 / 51개 (80%)</t>
+          <t>53 / 62개 (85%)</t>
         </is>
       </c>
     </row>
@@ -807,9 +807,24 @@
         </is>
       </c>
     </row>
+    <row r="34" ht="18" customHeight="1">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-13  ■■■■■■■  (14)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="18" customHeight="1">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-14  ■■■■■■■■  (16)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="32">
+  <mergeCells count="34">
     <mergeCell ref="A30:E30"/>
+    <mergeCell ref="A34:E34"/>
     <mergeCell ref="A24:E24"/>
     <mergeCell ref="A15:E15"/>
     <mergeCell ref="B6:E6"/>
@@ -834,6 +849,7 @@
     <mergeCell ref="A22:E22"/>
     <mergeCell ref="A17:E17"/>
     <mergeCell ref="A29:E29"/>
+    <mergeCell ref="A35:E35"/>
     <mergeCell ref="A20:E20"/>
     <mergeCell ref="A10:E10"/>
     <mergeCell ref="A28:E28"/>
@@ -852,7 +868,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1096,6 +1112,35 @@
       </c>
       <c r="E9" s="9" t="inlineStr">
         <is>
+          <t>완료</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="60" customHeight="1">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-09 ~ 05-15</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>입출고 v2 + 부서 결재</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>입출고 v2 4단계 마법사·멱등성·위저드 재디자인
+부서 결재 + 직원 권한 분리
+BOM 805건 입력 진행 + 부모 후보 추출
+재고 이미지 컬럼·데이터 모델 정리(legacy 제거)
+CI 안정화·개발 환경 정비</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="n">
+        <v>54</v>
+      </c>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
           <t>진행 중</t>
         </is>
       </c>
@@ -1111,7 +1156,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E52"/>
+  <dimension ref="A1:E63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1676,27 +1721,27 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="13" t="n">
+      <c r="A25" s="10" t="n">
         <v>24</v>
       </c>
-      <c r="B25" s="14" t="inlineStr">
+      <c r="B25" s="11" t="inlineStr">
         <is>
           <t>BOM 세팅 도구 (오프라인 · 848 품목)</t>
         </is>
       </c>
-      <c r="C25" s="13" t="inlineStr">
+      <c r="C25" s="10" t="inlineStr">
         <is>
           <t>BOM</t>
         </is>
       </c>
-      <c r="D25" s="15" t="inlineStr">
-        <is>
-          <t>🔲 예정</t>
-        </is>
-      </c>
-      <c r="E25" s="14" t="inlineStr">
-        <is>
-          <t>다음 주 마무리 + 실 데이터 입력</t>
+      <c r="D25" s="12" t="inlineStr">
+        <is>
+          <t>✅ 완료</t>
+        </is>
+      </c>
+      <c r="E25" s="11" t="inlineStr">
+        <is>
+          <t>805건 입력 진행 (튜닝 잔여)</t>
         </is>
       </c>
     </row>
@@ -1706,12 +1751,12 @@
       </c>
       <c r="B26" s="11" t="inlineStr">
         <is>
-          <t>자재 폼 ERP/옵션/모델 슬롯 편집</t>
+          <t>BOM 부모 후보 추출 스크립트</t>
         </is>
       </c>
       <c r="C26" s="10" t="inlineStr">
         <is>
-          <t>재고</t>
+          <t>BOM</t>
         </is>
       </c>
       <c r="D26" s="12" t="inlineStr">
@@ -1721,7 +1766,7 @@
       </c>
       <c r="E26" s="11" t="inlineStr">
         <is>
-          <t>ItemFormFields 공통화</t>
+          <t>입출고 관리대장 2024-2026 기반</t>
         </is>
       </c>
     </row>
@@ -1731,12 +1776,12 @@
       </c>
       <c r="B27" s="11" t="inlineStr">
         <is>
-          <t>부서간 재고 조정 4단계 위저드</t>
+          <t>자재 폼 ERP/옵션/모델 슬롯 편집</t>
         </is>
       </c>
       <c r="C27" s="10" t="inlineStr">
         <is>
-          <t>입출고</t>
+          <t>재고</t>
         </is>
       </c>
       <c r="D27" s="12" t="inlineStr">
@@ -1746,7 +1791,7 @@
       </c>
       <c r="E27" s="11" t="inlineStr">
         <is>
-          <t>흐름 재설계 시 재정리</t>
+          <t>ItemFormFields 공통화</t>
         </is>
       </c>
     </row>
@@ -1756,12 +1801,12 @@
       </c>
       <c r="B28" s="11" t="inlineStr">
         <is>
-          <t>주간 재고 변화 보고 화면</t>
+          <t>부서간 재고 조정 4단계 위저드</t>
         </is>
       </c>
       <c r="C28" s="10" t="inlineStr">
         <is>
-          <t>관리</t>
+          <t>입출고</t>
         </is>
       </c>
       <c r="D28" s="12" t="inlineStr">
@@ -1771,7 +1816,7 @@
       </c>
       <c r="E28" s="11" t="inlineStr">
         <is>
-          <t>공정별 입출고·달력 히스토리</t>
+          <t>입출고 v2에 흡수 정리</t>
         </is>
       </c>
     </row>
@@ -1781,12 +1826,12 @@
       </c>
       <c r="B29" s="11" t="inlineStr">
         <is>
-          <t>모바일 5탭 + 입출고 허브 (사전)</t>
+          <t>주간 재고 변화 보고 화면</t>
         </is>
       </c>
       <c r="C29" s="10" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>관리</t>
         </is>
       </c>
       <c r="D29" s="12" t="inlineStr">
@@ -1796,7 +1841,7 @@
       </c>
       <c r="E29" s="11" t="inlineStr">
         <is>
-          <t>최종 사용성은 후순위</t>
+          <t>공정별 입출고·달력 히스토리</t>
         </is>
       </c>
     </row>
@@ -1806,12 +1851,12 @@
       </c>
       <c r="B30" s="11" t="inlineStr">
         <is>
-          <t>공통 UI 컴포넌트 5종</t>
+          <t>모바일 5탭 + 입출고 허브 (사전)</t>
         </is>
       </c>
       <c r="C30" s="10" t="inlineStr">
         <is>
-          <t>인프라</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="D30" s="12" t="inlineStr">
@@ -1821,7 +1866,7 @@
       </c>
       <c r="E30" s="11" t="inlineStr">
         <is>
-          <t>FilterChip·SlidePanel·KpiCard 등</t>
+          <t>최종 사용성은 후순위</t>
         </is>
       </c>
     </row>
@@ -1831,12 +1876,12 @@
       </c>
       <c r="B31" s="11" t="inlineStr">
         <is>
-          <t>직원 명단 관리</t>
+          <t>공통 UI 컴포넌트 5종</t>
         </is>
       </c>
       <c r="C31" s="10" t="inlineStr">
         <is>
-          <t>직원</t>
+          <t>인프라</t>
         </is>
       </c>
       <c r="D31" s="12" t="inlineStr">
@@ -1844,7 +1889,11 @@
           <t>✅ 완료</t>
         </is>
       </c>
-      <c r="E31" s="11" t="inlineStr"/>
+      <c r="E31" s="11" t="inlineStr">
+        <is>
+          <t>FilterChip·SlidePanel·KpiCard 등</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="10" t="n">
@@ -1852,12 +1901,12 @@
       </c>
       <c r="B32" s="11" t="inlineStr">
         <is>
-          <t>부서별 담당 색상 배지 표시</t>
+          <t>입출고 v2 — 4단계 마법사</t>
         </is>
       </c>
       <c r="C32" s="10" t="inlineStr">
         <is>
-          <t>직원</t>
+          <t>입출고</t>
         </is>
       </c>
       <c r="D32" s="12" t="inlineStr">
@@ -1865,7 +1914,11 @@
           <t>✅ 완료</t>
         </is>
       </c>
-      <c r="E32" s="11" t="inlineStr"/>
+      <c r="E32" s="11" t="inlineStr">
+        <is>
+          <t>sub_type 분기 + 권한 가드 + 위저드 재디자인</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="10" t="n">
@@ -1873,12 +1926,12 @@
       </c>
       <c r="B33" s="11" t="inlineStr">
         <is>
-          <t>작업자 PIN 로그인 + 감사 이력</t>
+          <t>입출고 v2 — 중복 제출 방지(멱등성)</t>
         </is>
       </c>
       <c r="C33" s="10" t="inlineStr">
         <is>
-          <t>보안</t>
+          <t>입출고</t>
         </is>
       </c>
       <c r="D33" s="12" t="inlineStr">
@@ -1888,7 +1941,7 @@
       </c>
       <c r="E33" s="11" t="inlineStr">
         <is>
-          <t>수정 이력 자동 기록</t>
+          <t>client_request_id + 409/503 UX</t>
         </is>
       </c>
     </row>
@@ -1898,12 +1951,12 @@
       </c>
       <c r="B34" s="11" t="inlineStr">
         <is>
-          <t>로그인 및 권한 관리</t>
+          <t>입출고 내역 사람 친화 개선</t>
         </is>
       </c>
       <c r="C34" s="10" t="inlineStr">
         <is>
-          <t>보안</t>
+          <t>입출고</t>
         </is>
       </c>
       <c r="D34" s="12" t="inlineStr">
@@ -1913,7 +1966,7 @@
       </c>
       <c r="E34" s="11" t="inlineStr">
         <is>
-          <t>PIN 기반 — 역할별 접근 제어 예정</t>
+          <t>내 요청 카드·상세 표현·표 전면 개선</t>
         </is>
       </c>
     </row>
@@ -1923,12 +1976,12 @@
       </c>
       <c r="B35" s="11" t="inlineStr">
         <is>
-          <t>PC 화면 (데스크톱)</t>
+          <t>부서 결재 + 직원 권한 분리</t>
         </is>
       </c>
       <c r="C35" s="10" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>보안</t>
         </is>
       </c>
       <c r="D35" s="12" t="inlineStr">
@@ -1936,7 +1989,11 @@
           <t>✅ 완료</t>
         </is>
       </c>
-      <c r="E35" s="11" t="inlineStr"/>
+      <c r="E35" s="11" t="inlineStr">
+        <is>
+          <t>부서 결재 API 3건 + 조립 부서 담당 모델</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="10" t="n">
@@ -1944,12 +2001,12 @@
       </c>
       <c r="B36" s="11" t="inlineStr">
         <is>
-          <t>모바일 화면</t>
+          <t>재고 대시보드 품목 이미지 컬럼</t>
         </is>
       </c>
       <c r="C36" s="10" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>재고</t>
         </is>
       </c>
       <c r="D36" s="12" t="inlineStr">
@@ -1957,7 +2014,11 @@
           <t>✅ 완료</t>
         </is>
       </c>
-      <c r="E36" s="11" t="inlineStr"/>
+      <c r="E36" s="11" t="inlineStr">
+        <is>
+          <t>Next/Image 최적화</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="10" t="n">
@@ -1965,12 +2026,12 @@
       </c>
       <c r="B37" s="11" t="inlineStr">
         <is>
-          <t>다크 / 라이트 모드</t>
+          <t>데이터 모델 정리 (legacy 제거)</t>
         </is>
       </c>
       <c r="C37" s="10" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>인프라</t>
         </is>
       </c>
       <c r="D37" s="12" t="inlineStr">
@@ -1978,7 +2039,11 @@
           <t>✅ 완료</t>
         </is>
       </c>
-      <c r="E37" s="11" t="inlineStr"/>
+      <c r="E37" s="11" t="inlineStr">
+        <is>
+          <t>legacy_model + category + ShipPackage 제거</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="10" t="n">
@@ -1986,12 +2051,12 @@
       </c>
       <c r="B38" s="11" t="inlineStr">
         <is>
-          <t>관리자 화면</t>
+          <t>AppSelect 셀렉트 디자인 통일</t>
         </is>
       </c>
       <c r="C38" s="10" t="inlineStr">
         <is>
-          <t>관리</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="D38" s="12" t="inlineStr">
@@ -1999,7 +2064,11 @@
           <t>✅ 완료</t>
         </is>
       </c>
-      <c r="E38" s="11" t="inlineStr"/>
+      <c r="E38" s="11" t="inlineStr">
+        <is>
+          <t>공통 드롭다운 컴포넌트</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="10" t="n">
@@ -2007,12 +2076,12 @@
       </c>
       <c r="B39" s="11" t="inlineStr">
         <is>
-          <t>부서 관리 (DnD · 컬러 피커 · 검색)</t>
+          <t>로그인 단일 카드 화면</t>
         </is>
       </c>
       <c r="C39" s="10" t="inlineStr">
         <is>
-          <t>관리</t>
+          <t>보안</t>
         </is>
       </c>
       <c r="D39" s="12" t="inlineStr">
@@ -2020,7 +2089,11 @@
           <t>✅ 완료</t>
         </is>
       </c>
-      <c r="E39" s="11" t="inlineStr"/>
+      <c r="E39" s="11" t="inlineStr">
+        <is>
+          <t>3단계 → 콤보박스+PIN 1화면</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="10" t="n">
@@ -2028,7 +2101,7 @@
       </c>
       <c r="B40" s="11" t="inlineStr">
         <is>
-          <t>데이터 CSV 내보내기</t>
+          <t>관리자 화면 8섹션 + PIN</t>
         </is>
       </c>
       <c r="C40" s="10" t="inlineStr">
@@ -2041,7 +2114,11 @@
           <t>✅ 완료</t>
         </is>
       </c>
-      <c r="E40" s="11" t="inlineStr"/>
+      <c r="E40" s="11" t="inlineStr">
+        <is>
+          <t>BOM 가로분할·KPI 컴팩트화</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="10" t="n">
@@ -2049,12 +2126,12 @@
       </c>
       <c r="B41" s="11" t="inlineStr">
         <is>
-          <t>원클릭 실행 (start.bat)</t>
+          <t>생산 가능 수량 immediate/maximum</t>
         </is>
       </c>
       <c r="C41" s="10" t="inlineStr">
         <is>
-          <t>인프라</t>
+          <t>생산</t>
         </is>
       </c>
       <c r="D41" s="12" t="inlineStr">
@@ -2062,7 +2139,11 @@
           <t>✅ 완료</t>
         </is>
       </c>
-      <c r="E41" s="11" t="inlineStr"/>
+      <c r="E41" s="11" t="inlineStr">
+        <is>
+          <t>status 4분기 시각화</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="10" t="n">
@@ -2070,12 +2151,12 @@
       </c>
       <c r="B42" s="11" t="inlineStr">
         <is>
-          <t>테스트 자동화 (CI)</t>
+          <t>직원 명단 관리</t>
         </is>
       </c>
       <c r="C42" s="10" t="inlineStr">
         <is>
-          <t>인프라</t>
+          <t>직원</t>
         </is>
       </c>
       <c r="D42" s="12" t="inlineStr">
@@ -2083,11 +2164,7 @@
           <t>✅ 완료</t>
         </is>
       </c>
-      <c r="E42" s="11" t="inlineStr">
-        <is>
-          <t>pytest 42건 + vitest 12건</t>
-        </is>
-      </c>
+      <c r="E42" s="11" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="10" t="n">
@@ -2095,237 +2172,480 @@
       </c>
       <c r="B43" s="11" t="inlineStr">
         <is>
+          <t>부서별 담당 색상 배지 표시</t>
+        </is>
+      </c>
+      <c r="C43" s="10" t="inlineStr">
+        <is>
+          <t>직원</t>
+        </is>
+      </c>
+      <c r="D43" s="12" t="inlineStr">
+        <is>
+          <t>✅ 완료</t>
+        </is>
+      </c>
+      <c r="E43" s="11" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="10" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="11" t="inlineStr">
+        <is>
+          <t>작업자 PIN 로그인 + 감사 이력</t>
+        </is>
+      </c>
+      <c r="C44" s="10" t="inlineStr">
+        <is>
+          <t>보안</t>
+        </is>
+      </c>
+      <c r="D44" s="12" t="inlineStr">
+        <is>
+          <t>✅ 완료</t>
+        </is>
+      </c>
+      <c r="E44" s="11" t="inlineStr">
+        <is>
+          <t>수정 이력 자동 기록</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="10" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="11" t="inlineStr">
+        <is>
+          <t>로그인 및 권한 관리</t>
+        </is>
+      </c>
+      <c r="C45" s="10" t="inlineStr">
+        <is>
+          <t>보안</t>
+        </is>
+      </c>
+      <c r="D45" s="12" t="inlineStr">
+        <is>
+          <t>✅ 완료</t>
+        </is>
+      </c>
+      <c r="E45" s="11" t="inlineStr">
+        <is>
+          <t>PIN 기반 — 역할별 접근 제어 예정</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="10" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="11" t="inlineStr">
+        <is>
+          <t>PC 화면 (데스크톱)</t>
+        </is>
+      </c>
+      <c r="C46" s="10" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="D46" s="12" t="inlineStr">
+        <is>
+          <t>✅ 완료</t>
+        </is>
+      </c>
+      <c r="E46" s="11" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="10" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="11" t="inlineStr">
+        <is>
+          <t>모바일 화면</t>
+        </is>
+      </c>
+      <c r="C47" s="10" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="D47" s="12" t="inlineStr">
+        <is>
+          <t>✅ 완료</t>
+        </is>
+      </c>
+      <c r="E47" s="11" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="10" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="11" t="inlineStr">
+        <is>
+          <t>다크 / 라이트 모드</t>
+        </is>
+      </c>
+      <c r="C48" s="10" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="D48" s="12" t="inlineStr">
+        <is>
+          <t>✅ 완료</t>
+        </is>
+      </c>
+      <c r="E48" s="11" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="10" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="11" t="inlineStr">
+        <is>
+          <t>관리자 화면</t>
+        </is>
+      </c>
+      <c r="C49" s="10" t="inlineStr">
+        <is>
+          <t>관리</t>
+        </is>
+      </c>
+      <c r="D49" s="12" t="inlineStr">
+        <is>
+          <t>✅ 완료</t>
+        </is>
+      </c>
+      <c r="E49" s="11" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="10" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="11" t="inlineStr">
+        <is>
+          <t>부서 관리 (DnD · 컬러 피커 · 검색)</t>
+        </is>
+      </c>
+      <c r="C50" s="10" t="inlineStr">
+        <is>
+          <t>관리</t>
+        </is>
+      </c>
+      <c r="D50" s="12" t="inlineStr">
+        <is>
+          <t>✅ 완료</t>
+        </is>
+      </c>
+      <c r="E50" s="11" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="10" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="11" t="inlineStr">
+        <is>
+          <t>데이터 CSV 내보내기</t>
+        </is>
+      </c>
+      <c r="C51" s="10" t="inlineStr">
+        <is>
+          <t>관리</t>
+        </is>
+      </c>
+      <c r="D51" s="12" t="inlineStr">
+        <is>
+          <t>✅ 완료</t>
+        </is>
+      </c>
+      <c r="E51" s="11" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="10" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" s="11" t="inlineStr">
+        <is>
+          <t>원클릭 실행 (start.bat)</t>
+        </is>
+      </c>
+      <c r="C52" s="10" t="inlineStr">
+        <is>
+          <t>인프라</t>
+        </is>
+      </c>
+      <c r="D52" s="12" t="inlineStr">
+        <is>
+          <t>✅ 완료</t>
+        </is>
+      </c>
+      <c r="E52" s="11" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="10" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" s="11" t="inlineStr">
+        <is>
+          <t>테스트 자동화 (CI)</t>
+        </is>
+      </c>
+      <c r="C53" s="10" t="inlineStr">
+        <is>
+          <t>인프라</t>
+        </is>
+      </c>
+      <c r="D53" s="12" t="inlineStr">
+        <is>
+          <t>✅ 완료</t>
+        </is>
+      </c>
+      <c r="E53" s="11" t="inlineStr">
+        <is>
+          <t>pytest 42건 + vitest 12건</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="10" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" s="11" t="inlineStr">
+        <is>
           <t>WAL-safe 백업 / 복구</t>
         </is>
       </c>
-      <c r="C43" s="10" t="inlineStr">
+      <c r="C54" s="10" t="inlineStr">
         <is>
           <t>인프라</t>
         </is>
       </c>
-      <c r="D43" s="12" t="inlineStr">
+      <c r="D54" s="12" t="inlineStr">
         <is>
           <t>✅ 완료</t>
         </is>
       </c>
-      <c r="E43" s="11" t="inlineStr">
+      <c r="E54" s="11" t="inlineStr">
         <is>
           <t>ops 스크립트 자동화</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="13" t="n">
-        <v>43</v>
-      </c>
-      <c r="B44" s="14" t="inlineStr">
+    <row r="55">
+      <c r="A55" s="13" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" s="14" t="inlineStr">
         <is>
           <t>입출고 화면·내역 흐름 재설계</t>
         </is>
       </c>
-      <c r="C44" s="13" t="inlineStr">
+      <c r="C55" s="13" t="inlineStr">
         <is>
           <t>입출고</t>
         </is>
       </c>
-      <c r="D44" s="15" t="inlineStr">
+      <c r="D55" s="15" t="inlineStr">
         <is>
           <t>🔲 예정</t>
         </is>
       </c>
-      <c r="E44" s="14" t="inlineStr">
+      <c r="E55" s="14" t="inlineStr">
         <is>
           <t>담당자 동선 분석 후 (다음 주~다다음주)</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="13" t="n">
-        <v>44</v>
-      </c>
-      <c r="B45" s="14" t="inlineStr">
+    <row r="56">
+      <c r="A56" s="13" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" s="14" t="inlineStr">
         <is>
           <t>실 재고 데이터 입력 + 직원 테스트</t>
         </is>
       </c>
-      <c r="C45" s="13" t="inlineStr">
+      <c r="C56" s="13" t="inlineStr">
         <is>
           <t>데이터</t>
         </is>
       </c>
-      <c r="D45" s="15" t="inlineStr">
+      <c r="D56" s="15" t="inlineStr">
         <is>
           <t>🔲 예정</t>
         </is>
       </c>
-      <c r="E45" s="14" t="inlineStr">
+      <c r="E56" s="14" t="inlineStr">
         <is>
           <t>BOM·입출고 정리 후</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="13" t="n">
-        <v>45</v>
-      </c>
-      <c r="B46" s="14" t="inlineStr">
+    <row r="57">
+      <c r="A57" s="13" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" s="14" t="inlineStr">
         <is>
           <t>역할별 접근 권한 연동</t>
         </is>
       </c>
-      <c r="C46" s="13" t="inlineStr">
+      <c r="C57" s="13" t="inlineStr">
         <is>
           <t>보안</t>
         </is>
       </c>
-      <c r="D46" s="15" t="inlineStr">
+      <c r="D57" s="15" t="inlineStr">
         <is>
           <t>🔲 예정</t>
         </is>
       </c>
-      <c r="E46" s="14" t="inlineStr">
+      <c r="E57" s="14" t="inlineStr">
         <is>
           <t>부서·역할 기반 (PIN 로그인 완료)</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="13" t="n">
-        <v>46</v>
-      </c>
-      <c r="B47" s="14" t="inlineStr">
+    <row r="58">
+      <c r="A58" s="13" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" s="14" t="inlineStr">
         <is>
           <t>총재고 / 가용재고 / 예약재고 분리</t>
         </is>
       </c>
-      <c r="C47" s="13" t="inlineStr">
+      <c r="C58" s="13" t="inlineStr">
         <is>
           <t>재고</t>
         </is>
       </c>
-      <c r="D47" s="15" t="inlineStr">
+      <c r="D58" s="15" t="inlineStr">
         <is>
           <t>🔲 예정</t>
         </is>
       </c>
-      <c r="E47" s="14" t="inlineStr">
+      <c r="E58" s="14" t="inlineStr">
         <is>
           <t>재고 가용성 계산 고도화</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="13" t="n">
-        <v>47</v>
-      </c>
-      <c r="B48" s="14" t="inlineStr">
+    <row r="59">
+      <c r="A59" s="13" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" s="14" t="inlineStr">
         <is>
           <t>외부 접근 환경 구성</t>
         </is>
       </c>
-      <c r="C48" s="13" t="inlineStr">
+      <c r="C59" s="13" t="inlineStr">
         <is>
           <t>인프라</t>
         </is>
       </c>
-      <c r="D48" s="15" t="inlineStr">
+      <c r="D59" s="15" t="inlineStr">
         <is>
           <t>🔲 예정</t>
         </is>
       </c>
-      <c r="E48" s="14" t="inlineStr">
+      <c r="E59" s="14" t="inlineStr">
         <is>
           <t>PC 또는 NAS 서버 + API 인증</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="13" t="n">
-        <v>48</v>
-      </c>
-      <c r="B49" s="14" t="inlineStr">
+    <row r="60">
+      <c r="A60" s="13" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" s="14" t="inlineStr">
         <is>
           <t>발주 관리</t>
         </is>
       </c>
-      <c r="C49" s="13" t="inlineStr">
+      <c r="C60" s="13" t="inlineStr">
         <is>
           <t>구매</t>
         </is>
       </c>
-      <c r="D49" s="15" t="inlineStr">
+      <c r="D60" s="15" t="inlineStr">
         <is>
           <t>🔲 예정</t>
         </is>
       </c>
-      <c r="E49" s="14" t="inlineStr"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="13" t="n">
-        <v>49</v>
-      </c>
-      <c r="B50" s="14" t="inlineStr">
+      <c r="E60" s="14" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="13" t="n">
+        <v>60</v>
+      </c>
+      <c r="B61" s="14" t="inlineStr">
         <is>
           <t>생산 실적 / 원가 관리</t>
         </is>
       </c>
-      <c r="C50" s="13" t="inlineStr">
+      <c r="C61" s="13" t="inlineStr">
         <is>
           <t>생산</t>
         </is>
       </c>
-      <c r="D50" s="15" t="inlineStr">
+      <c r="D61" s="15" t="inlineStr">
         <is>
           <t>🔲 예정</t>
         </is>
       </c>
-      <c r="E50" s="14" t="inlineStr"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="13" t="n">
-        <v>50</v>
-      </c>
-      <c r="B51" s="14" t="inlineStr">
+      <c r="E61" s="14" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="13" t="n">
+        <v>61</v>
+      </c>
+      <c r="B62" s="14" t="inlineStr">
         <is>
           <t>부서별 생산진행도 대시보드</t>
         </is>
       </c>
-      <c r="C51" s="13" t="inlineStr">
+      <c r="C62" s="13" t="inlineStr">
         <is>
           <t>관리</t>
         </is>
       </c>
-      <c r="D51" s="15" t="inlineStr">
+      <c r="D62" s="15" t="inlineStr">
         <is>
           <t>🔲 예정</t>
         </is>
       </c>
-      <c r="E51" s="14" t="inlineStr">
+      <c r="E62" s="14" t="inlineStr">
         <is>
           <t>사장님 요청 — 검토 중</t>
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="13" t="n">
-        <v>51</v>
-      </c>
-      <c r="B52" s="14" t="inlineStr">
+    <row r="63">
+      <c r="A63" s="13" t="n">
+        <v>62</v>
+      </c>
+      <c r="B63" s="14" t="inlineStr">
         <is>
           <t>출하 거래처 관리</t>
         </is>
       </c>
-      <c r="C52" s="13" t="inlineStr">
+      <c r="C63" s="13" t="inlineStr">
         <is>
           <t>출하</t>
         </is>
       </c>
-      <c r="D52" s="15" t="inlineStr">
+      <c r="D63" s="15" t="inlineStr">
         <is>
           <t>🔲 예정</t>
         </is>
       </c>
-      <c r="E52" s="14" t="inlineStr">
+      <c r="E63" s="14" t="inlineStr">
         <is>
           <t>거래처 마스터 + 출하 이력</t>
         </is>
@@ -2342,7 +2662,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D26"/>
+  <dimension ref="A1:D28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2958,6 +3278,54 @@
         </is>
       </c>
       <c r="D26" s="16" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="50" customHeight="1">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="n">
+        <v>14</v>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-13 backend+frontend: 부서 결재 + 직원 권한 분리
+2026-05-13 frontend: 입출고 v2 UX 개선
+2026-05-13 docs+dev: 주간보고/개발현황/ONBOARDING 갱신 + BOM 부모 추출 스크립
+2026-05-13 data: 입출고 관리대장 원본(2024-2026) + BOM 부모 후보 추출본
+2026-05-13 fix: openapi baseline 갱신 (부서 결재 엔드포인트 3건)</t>
+        </is>
+      </c>
+      <c r="D27" s="7" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="50" customHeight="1">
+      <c r="A28" s="16" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B28" s="16" t="n">
+        <v>16</v>
+      </c>
+      <c r="C28" s="17" t="inlineStr">
+        <is>
+          <t>2026-05-14 frontend: 입출고 v2 위저드 시각 재디자인 (Step 2/3/4 + 카트)
+2026-05-14 frontend: 입출고 v2 BOM 묶음 헤더 통합 + 최종확인 1단 + 표 스크롤 보
+2026-05-14 refactor: 완제품 출하(ship) 작업유형 + ShipPackage 전체 제거
+2026-05-14 fix: DesktopInventoryView 미커밋 이미지 manifest 의존 제거
+2026-05-14 frontend: 재고 대시보드 품목 이미지 컬럼 추가</t>
+        </is>
+      </c>
+      <c r="D28" s="16" t="inlineStr">
         <is>
           <t>Frontend</t>
         </is>
@@ -2974,7 +3342,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D392"/>
+  <dimension ref="A1:D422"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11607,6 +11975,666 @@
         </is>
       </c>
     </row>
+    <row r="393">
+      <c r="A393" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B393" s="7" t="inlineStr">
+        <is>
+          <t>6661fb9</t>
+        </is>
+      </c>
+      <c r="C393" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-13 backend+frontend: 부서 결재 + 직원 권한 분리</t>
+        </is>
+      </c>
+      <c r="D393" s="7" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" s="16" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B394" s="16" t="inlineStr">
+        <is>
+          <t>46874a4</t>
+        </is>
+      </c>
+      <c r="C394" s="17" t="inlineStr">
+        <is>
+          <t>2026-05-13 frontend: 입출고 v2 UX 개선</t>
+        </is>
+      </c>
+      <c r="D394" s="16" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B395" s="7" t="inlineStr">
+        <is>
+          <t>b440c01</t>
+        </is>
+      </c>
+      <c r="C395" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-13 docs+dev: 주간보고/개발현황/ONBOARDING 갱신 + BOM 부모 추출 스크립트</t>
+        </is>
+      </c>
+      <c r="D395" s="7" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" s="16" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B396" s="16" t="inlineStr">
+        <is>
+          <t>5ce4ca0</t>
+        </is>
+      </c>
+      <c r="C396" s="17" t="inlineStr">
+        <is>
+          <t>2026-05-13 data: 입출고 관리대장 원본(2024-2026) + BOM 부모 후보 추출본</t>
+        </is>
+      </c>
+      <c r="D396" s="16" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B397" s="7" t="inlineStr">
+        <is>
+          <t>f177f80</t>
+        </is>
+      </c>
+      <c r="C397" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-13 fix: openapi baseline 갱신 (부서 결재 엔드포인트 3건)</t>
+        </is>
+      </c>
+      <c r="D397" s="7" t="inlineStr">
+        <is>
+          <t>fix</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" s="16" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B398" s="16" t="inlineStr">
+        <is>
+          <t>45c4de7</t>
+        </is>
+      </c>
+      <c r="C398" s="17" t="inlineStr">
+        <is>
+          <t>2026-05-13 docs: 사내 발표용 HTML 슬라이드 데크 (DEXCOWIN MES 9장)</t>
+        </is>
+      </c>
+      <c r="D398" s="16" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B399" s="7" t="inlineStr">
+        <is>
+          <t>bdb9da9</t>
+        </is>
+      </c>
+      <c r="C399" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-13 frontend: 사이드바 메뉴 재클릭 시 페이지 기본 상태 리셋</t>
+        </is>
+      </c>
+      <c r="D399" s="7" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" s="16" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B400" s="16" t="inlineStr">
+        <is>
+          <t>57cb37d</t>
+        </is>
+      </c>
+      <c r="C400" s="17" t="inlineStr">
+        <is>
+          <t>2026-05-13 backend+frontend: 조립 부서 직원 담당 모델 등록 + 입출고 조립 그룹 우선 정렬</t>
+        </is>
+      </c>
+      <c r="D400" s="16" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B401" s="7" t="inlineStr">
+        <is>
+          <t>bb8593e</t>
+        </is>
+      </c>
+      <c r="C401" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-13 frontend+backend: 내 요청 카드 재설계 + 입출고 내역 상세 사람 친화화</t>
+        </is>
+      </c>
+      <c r="D401" s="7" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" s="16" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B402" s="16" t="inlineStr">
+        <is>
+          <t>1629d3e</t>
+        </is>
+      </c>
+      <c r="C402" s="17" t="inlineStr">
+        <is>
+          <t>2026-05-13 docs: gitignore 루트 임시 산출물 패턴 추가 (step*.png, v*.png, verify_out.log)</t>
+        </is>
+      </c>
+      <c r="D402" s="16" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B403" s="7" t="inlineStr">
+        <is>
+          <t>ecaec3a</t>
+        </is>
+      </c>
+      <c r="C403" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-13 frontend: 입출고 v2 위저드 카드 동적 높이 + 섹션 탭 재디자인</t>
+        </is>
+      </c>
+      <c r="D403" s="7" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" s="16" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B404" s="16" t="inlineStr">
+        <is>
+          <t>e104ebb</t>
+        </is>
+      </c>
+      <c r="C404" s="17" t="inlineStr">
+        <is>
+          <t>2026-05-13 data: BOM 부모 후보 + 세팅 도구 산출물 갱신</t>
+        </is>
+      </c>
+      <c r="D404" s="16" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B405" s="7" t="inlineStr">
+        <is>
+          <t>5f90e6b</t>
+        </is>
+      </c>
+      <c r="C405" s="8" t="inlineStr">
+        <is>
+          <t>fix: IoComposeView useLayoutEffect ref capture</t>
+        </is>
+      </c>
+      <c r="D405" s="7" t="inlineStr">
+        <is>
+          <t>fix</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" s="16" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B406" s="16" t="inlineStr">
+        <is>
+          <t>eba8371</t>
+        </is>
+      </c>
+      <c r="C406" s="17" t="inlineStr">
+        <is>
+          <t>frontend: 입출고 v2 단계 카드 높이 보정</t>
+        </is>
+      </c>
+      <c r="D406" s="16" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B407" s="7" t="inlineStr">
+        <is>
+          <t>b574cda</t>
+        </is>
+      </c>
+      <c r="C407" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-14 frontend: 입출고 v2 위저드 시각 재디자인 (Step 2/3/4 + 카트)</t>
+        </is>
+      </c>
+      <c r="D407" s="7" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" s="16" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B408" s="16" t="inlineStr">
+        <is>
+          <t>44ceeb1</t>
+        </is>
+      </c>
+      <c r="C408" s="17" t="inlineStr">
+        <is>
+          <t>2026-05-14 frontend: 입출고 v2 BOM 묶음 헤더 통합 + 최종확인 1단 + 표 스크롤 보존 시도(미해결)</t>
+        </is>
+      </c>
+      <c r="D408" s="16" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B409" s="7" t="inlineStr">
+        <is>
+          <t>c545bfa</t>
+        </is>
+      </c>
+      <c r="C409" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-14 refactor: 완제품 출하(ship) 작업유형 + ShipPackage 전체 제거</t>
+        </is>
+      </c>
+      <c r="D409" s="7" t="inlineStr">
+        <is>
+          <t>refactor</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" s="16" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B410" s="16" t="inlineStr">
+        <is>
+          <t>112c56d</t>
+        </is>
+      </c>
+      <c r="C410" s="17" t="inlineStr">
+        <is>
+          <t>2026-05-14 fix: DesktopInventoryView 미커밋 이미지 manifest 의존 제거</t>
+        </is>
+      </c>
+      <c r="D410" s="16" t="inlineStr">
+        <is>
+          <t>fix</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B411" s="7" t="inlineStr">
+        <is>
+          <t>f4229a9</t>
+        </is>
+      </c>
+      <c r="C411" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-14 frontend: 재고 대시보드 품목 이미지 컬럼 추가</t>
+        </is>
+      </c>
+      <c r="D411" s="7" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" s="16" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B412" s="16" t="inlineStr">
+        <is>
+          <t>97943a3</t>
+        </is>
+      </c>
+      <c r="C412" s="17" t="inlineStr">
+        <is>
+          <t>2026-05-14 frontend: 입출고 v2 draft 카드 헤더 모든 번들 표시 + 부모 수량</t>
+        </is>
+      </c>
+      <c r="D412" s="16" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B413" s="7" t="inlineStr">
+        <is>
+          <t>b797e96</t>
+        </is>
+      </c>
+      <c r="C413" s="8" t="inlineStr">
+        <is>
+          <t>fix: InventoryItemRow img → next/image Image 컴포넌트로 변경</t>
+        </is>
+      </c>
+      <c r="D413" s="7" t="inlineStr">
+        <is>
+          <t>fix</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" s="16" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B414" s="16" t="inlineStr">
+        <is>
+          <t>e498de4</t>
+        </is>
+      </c>
+      <c r="C414" s="17" t="inlineStr">
+        <is>
+          <t>2026-05-14 docs: gitignore에 품목 이미지 추출 원본 폴더 제외 추가</t>
+        </is>
+      </c>
+      <c r="D414" s="16" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B415" s="7" t="inlineStr">
+        <is>
+          <t>78b16d6</t>
+        </is>
+      </c>
+      <c r="C415" s="8" t="inlineStr">
+        <is>
+          <t>fix: 재고 대시보드 이미지 컬럼 안 뜨는 문제 해결</t>
+        </is>
+      </c>
+      <c r="D415" s="7" t="inlineStr">
+        <is>
+          <t>fix</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" s="16" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B416" s="16" t="inlineStr">
+        <is>
+          <t>1d00169</t>
+        </is>
+      </c>
+      <c r="C416" s="17" t="inlineStr">
+        <is>
+          <t>2026-05-14 refactor: legacy_model 필드 완전 제거 (DB + API + UI)</t>
+        </is>
+      </c>
+      <c r="D416" s="16" t="inlineStr">
+        <is>
+          <t>refactor</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B417" s="7" t="inlineStr">
+        <is>
+          <t>3f7e67c</t>
+        </is>
+      </c>
+      <c r="C417" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-14 docs: 멀티에이전트 시스템 추가 (CEO/Frontend/Backend/QA)</t>
+        </is>
+      </c>
+      <c r="D417" s="7" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" s="16" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B418" s="16" t="inlineStr">
+        <is>
+          <t>2ba5b57</t>
+        </is>
+      </c>
+      <c r="C418" s="17" t="inlineStr">
+        <is>
+          <t>2026-05-14 docs: 티먹스 멀티에이전트 파일 제거</t>
+        </is>
+      </c>
+      <c r="D418" s="16" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B419" s="7" t="inlineStr">
+        <is>
+          <t>2ae3ed6</t>
+        </is>
+      </c>
+      <c r="C419" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-14 refactor: 폐기된 category 컬럼 잔재 정리 (좀비 스크립트 archive, process_type_code 통일)</t>
+        </is>
+      </c>
+      <c r="D419" s="7" t="inlineStr">
+        <is>
+          <t>refactor</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" s="16" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B420" s="16" t="inlineStr">
+        <is>
+          <t>e77bd15</t>
+        </is>
+      </c>
+      <c r="C420" s="17" t="inlineStr">
+        <is>
+          <t>2026-05-14 desktop: 입출고 내역 표 전면 개선</t>
+        </is>
+      </c>
+      <c r="D420" s="16" t="inlineStr">
+        <is>
+          <t>desktop</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B421" s="7" t="inlineStr">
+        <is>
+          <t>5c7c0a1</t>
+        </is>
+      </c>
+      <c r="C421" s="8" t="inlineStr">
+        <is>
+          <t>fix: CI 실패 2건 수정 (Vitest 라벨 기대값, OpenAPI drift)</t>
+        </is>
+      </c>
+      <c r="D421" s="7" t="inlineStr">
+        <is>
+          <t>fix</t>
+        </is>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" s="16" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B422" s="16" t="inlineStr">
+        <is>
+          <t>21454cb</t>
+        </is>
+      </c>
+      <c r="C422" s="17" t="inlineStr">
+        <is>
+          <t>docs: 발표자료 인터뷰 기반 전면 재작성 (9슬라이드)</t>
+        </is>
+      </c>
+      <c r="D422" s="16" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>